<commit_message>
Memperbaiki fungsi keanggotaan pelayanan dan harga
</commit_message>
<xml_diff>
--- a/peringkat.xlsx
+++ b/peringkat.xlsx
@@ -452,13 +452,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="B2" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C2" t="n">
-        <v>34513</v>
+        <v>22360</v>
       </c>
       <c r="D2" t="n">
         <v>90</v>
@@ -466,13 +466,13 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B3" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C3" t="n">
-        <v>22360</v>
+        <v>22012</v>
       </c>
       <c r="D3" t="n">
         <v>90</v>
@@ -480,13 +480,13 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B4" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C4" t="n">
-        <v>22012</v>
+        <v>27315</v>
       </c>
       <c r="D4" t="n">
         <v>90</v>
@@ -494,13 +494,13 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="B5" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" t="n">
-        <v>27315</v>
+        <v>24551</v>
       </c>
       <c r="D5" t="n">
         <v>90</v>
@@ -508,13 +508,13 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="B6" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C6" t="n">
-        <v>24551</v>
+        <v>29811</v>
       </c>
       <c r="D6" t="n">
         <v>90</v>

</xml_diff>